<commit_message>
DC: port dcsim-site work since the merge (Zabbix/NetBox available, clips, bright-room stills, lights-off hero) + 2026-10-15 decisions (Design license line, Excel export and device picker shipped, template v1.3, no public demo, new example workbook)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/dc/downloads/dc-import-template.xlsx
+++ b/public/dc/downloads/dc-import-template.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Devices" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cables" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Racks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Networks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cooling" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readings" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Racks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Networks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cooling" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CustomDevices" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readings" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -298,37 +300,17 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Same rack names as in Devices</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Row name. Racks in the same row stand side by side</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Order in the row: 1, 2, 3 …</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Default 42</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>19 (default) or 10 for a mini rack</t>
+        <t>Room name used in Racks.row names or Cooling.serves, e.g. "Hall 1"</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Aisle the rack front faces: A or B. Empty = rows alternate automatically (hot/cold aisle)</t>
+        <t>Installed lighting load in W (default 6 W/m² × area). Lights-off mode shows the saving</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Design power for this rack, if known</t>
+        <t>e.g. Europe/Warsaw — used by Lights auto</t>
       </text>
     </comment>
   </commentList>
@@ -343,57 +325,42 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Utility feed, generator, UPS, panel, breaker or PDU. If it is mounted in a rack, also list it in Devices with the same name</t>
+        <t>Same rack names as in Devices</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>utility, wall outlet, generator, UPS, panel, breaker, PDU, power strip, smart plug</t>
+        <t>Row name. Racks in the same row stand side by side</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Number with unit: 11 kVA, 16 A, 22 kW</t>
+        <t>Room name from the Rooms sheet (one room if empty)</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Name of the item above it in the chain</t>
+        <t>Order in the row: 1, 2, 3 …</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Feed letter: A or B</t>
+        <t>Default 42</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Rack it sits in or supplies (for PDUs)</t>
+        <t>19 (default) or 10 for a mini rack</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>e.g. 230 V, 400 V, 120 V</t>
+        <t>Aisle the rack front faces: A or B. Empty = rows alternate automatically (hot/cold aisle)</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>1 or 3</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>For single-phase items fed from a 3-phase supply: L1, L2 or L3</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>UPS only: runtime in minutes at the load you expect (from the vendor table)</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>UPS / battery cabinet only: usable battery energy in kWh</t>
+        <t>Design power for this rack, if known</t>
       </text>
     </comment>
   </commentList>
@@ -408,17 +375,57 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>VLAN id</t>
+        <t>Utility feed, generator, UPS, panel, breaker or PDU. If it is mounted in a rack, also list it in Devices with the same name</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>utility, wall outlet, generator, UPS, panel, breaker, PDU, power strip, smart plug</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>servers, storage, management, IoT, guest, AI fabric …</t>
+        <t>Number with unit: 11 kVA, 16 A, 22 kW</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Optional, e.g. 10.0.10.0/24</t>
+        <t>Name of the item above it in the chain</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Feed letter: A or B</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Rack it sits in or supplies (for PDUs)</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. 230 V, 400 V, 120 V</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>1 or 3</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>For single-phase items fed from a 3-phase supply: L1, L2 or L3</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>UPS only: runtime in minutes at the load you expect (from the vendor table)</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>UPS / battery cabinet only: usable battery energy in kWh</t>
       </text>
     </comment>
   </commentList>
@@ -431,19 +438,19 @@
     <author>template</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>CRAH, CRAC, in-row, rear-door, CDU, split AC</t>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>VLAN id</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Cooling capacity</t>
+        <t>servers, storage, management, IoT, guest, AI fabric …</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Rows or racks it cools, separated by ;</t>
+        <t>Optional, e.g. 10.0.10.0/24</t>
       </text>
     </comment>
   </commentList>
@@ -451,6 +458,81 @@
 </file>
 
 <file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>template</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>CRAH, CRAC, in-row, rear-door, CDU, split AC</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Cooling capacity</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Rows or racks it cools, separated by ;</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Short name you then use in Devices.model, e.g. "my-nas"</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>server, gpu_server, switch, storage, nas, mini_pc, sbc, patch_panel, pdu, ups, rack, crah, cdu, fire, generic …</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Empty = no U (shelf)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>19 (default) or 10</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Rating of one PSU</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>front-to-back, back-to-front, side, none</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. "2x25G SFP28; 4x1G RJ45; 1x IPMI"</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Category fields as JSON, e.g. {"va":1500,"runtime":[{"load_w":500,"minutes":12}]}</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>template</author>
@@ -769,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -809,81 +891,218 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSV works too: one file per sheet (devices.csv, cables.csv, racks.csv, power.csv, networks.csv, cooling.csv, readings.csv) with the same column names.</t>
+          <t>Template v1.2 (2026-10-14): optional CustomDevices sheet — describe a device we do not know, then use its name in Devices.model.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Template v1.3 (2026-10-15): optional Rooms sheet (size, lighting_w, timezone) and Racks.room.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CSV works too: one file per sheet (devices.csv, cables.csv, racks.csv, power.csv, networks.csv, cooling.csv, customdevices.csv, readings.csv) with the same column names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Devices — what sits where. From the model name we fill in size, weight, power, airflow and the inside of the device.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Cables — every power, network and storage cable, end to end. Enables the Cabling view (trace any cable), the Power view and the Network view.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Racks — which racks stand in which row. Without it, all racks from Devices are placed in one row.</t>
+          <t>Devices — what sits where. From the model name we fill in size, weight, power, airflow and the inside of the device.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Power — utility, UPS, panels, breakers and PDUs. Enables the power diagram, "what if feed A fails" and overload checks.</t>
+          <t>Cables — every power, network and storage cable, end to end. Enables the Cabling view (trace any cable), the Power view and the Network view.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Networks — your VLANs. Colours links in the Network view.</t>
+          <t>Racks — which racks stand in which row. Without it, all racks from Devices are placed in one row.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cooling — air conditioning and liquid cooling. Enables cooling-vs-heat checks and "what if AC-1 stops".</t>
+          <t>Power — utility, UPS, panels, breakers and PDUs. Enables the power diagram, "what if feed A fails" and overload checks.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Readings — history exported from your monitoring tool (Zabbix, SolarWinds, PRTG, Grafana …). Makes the simulation match your real room.</t>
+          <t>Networks — your VLANs. Colours links in the Network view.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cooling — air conditioning and liquid cooling. Enables cooling-vs-heat checks and "what if AC-1 stops".</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Readings — history exported from your monitoring tool (Zabbix, SolarWinds, PRTG, Grafana …). Makes the simulation match your real room.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Unknown model names are fine: they become a plain box of the right height and you can identify them later.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-01 14:00</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>pve-01</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>power_w</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-01 14:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>PDU-R01-A</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>current_a</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-01 14:00</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>sw-core:SFP+1</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>link_mbps</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-01 14:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>R01</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>inlet_temp_c</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>24.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1639,7 +1858,95 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>room</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>length_m</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>width_m</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>height_m</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>raised_floor_mm</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>lighting_w</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>timezone</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Hall 1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>580</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Europe/Warsaw</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1647,8 +1954,9 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1662,27 +1970,32 @@
           <t>row</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>room</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>position</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>height_u</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>width_in</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>front_faces</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>max_kw</t>
         </is>
@@ -1699,21 +2012,26 @@
           <t>Row A</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Hall 1</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="F2" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="H2" s="5" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1728,21 +2046,26 @@
           <t>Row A</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Hall 1</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="F3" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="H3" s="5" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1757,27 +2080,32 @@
           <t>Row B</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Hall 1</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="F4" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="H4" s="5" t="n">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A,B"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1786,7 +2114,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2116,7 +2444,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2207,7 +2535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2282,121 +2610,186 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>time</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>item</t>
+          <t>category</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>brand</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>height_u</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>width_in</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>depth_mm</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>weight_kg</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>psu_count</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>psu_w</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>idle_w</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>typical_w</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>max_w</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>airflow</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>inlet_max_c</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>ports</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>extra_json</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01 14:00</t>
+          <t>my-nas</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>pve-01</t>
+          <t>nas</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>power_w</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-01 14:00</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>PDU-R01-A</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>current_a</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-01 14:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>sw-core:SFP+1</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>link_mbps</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-01 14:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>R01</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>inlet_temp_c</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>24.5</v>
+          <t>Acme</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>NAS-8</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>front-to-back</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>2x10G SFP+; 2x1G RJ45</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>{"bays":"8x3.5"}</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DC: /dc/world/ — famous data centers on an interactive earth (globe.gl, site-only code): 100 sites, 25 estates, cut a link / lose a site, compare two sites, where's my data center, Map/Photo earth, URL state; one page per site and estate with build-time maps, open dataset page (CC BY 4.0); dc-world sync script. Estate on /dc/: optional HeroStage view (appears when state-dc-estate clips exist) + 'whole estate on one earth' section. Template v1.4 (Sites, Links; Rooms available).
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/dc/downloads/dc-import-template.xlsx
+++ b/public/dc/downloads/dc-import-template.xlsx
@@ -10,13 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Devices" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cables" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Racks" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Networks" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cooling" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CustomDevices" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readings" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sites" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Racks" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Networks" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Links" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cooling" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CustomDevices" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readings" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -227,6 +229,86 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Short name you then use in Devices.model, e.g. "my-nas"</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>server, gpu_server, switch, storage, nas, mini_pc, sbc, patch_panel, pdu, ups, rack, crah, cdu, fire, generic …</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Empty = no U (shelf)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>19 (default) or 10</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Rating of one PSU</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>front-to-back, back-to-front, side, none</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. "2x25G SFP28; 4x1G RJ45; 1x IPMI"</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Category fields as JSON, e.g. {"va":1500,"runtime":[{"load_w":500,"minutes":12}]}</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Date and time, e.g. 2026-10-01 14:00</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Device, rack, power item or sensor name; for a port use device:port, e.g. sw-core:SFP+1</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>power_w, current_a, inlet_temp_c, outlet_temp_c, humidity_pct, link_mbps, port_errors, gpu_util_pct, tokens_per_s …</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Number</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -300,17 +382,47 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Room name used in Racks.row names or Cooling.serves, e.g. "Hall 1"</t>
+        <t>Site name used in Rooms.site and Links, e.g. "FRA-1"</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>ISO 3166 two letters, e.g. DE</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Decimal degrees, e.g. 50.1109 (negative = south)</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Decimal degrees, e.g. 8.6821 (negative = west)</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Installed lighting load in W (default 6 W/m² × area). Lights-off mode shows the saving</t>
+        <t>e.g. Europe/Berlin — used by Lights auto and the globe day/night</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>e.g. Europe/Warsaw — used by Lights auto</t>
+        <t>primary, dr, edge, colo, cloud</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Operator or colo provider, free text</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Design IT load in kW for sites without a modelled hall</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Design PUE for sites without a modelled hall</t>
       </text>
     </comment>
   </commentList>
@@ -325,42 +437,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Same rack names as in Devices</t>
+        <t>Room name used in Racks.row names or Cooling.serves, e.g. "Hall 1"</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Row name. Racks in the same row stand side by side</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Room name from the Rooms sheet (one room if empty)</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Order in the row: 1, 2, 3 …</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Default 42</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>19 (default) or 10 for a mini rack</t>
+        <t>Site name from the Sites sheet (one site if empty)</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Aisle the rack front faces: A or B. Empty = rows alternate automatically (hot/cold aisle)</t>
+        <t>Installed lighting load in W (default 6 W/m² × area). Lights-off mode shows the saving</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Design power for this rack, if known</t>
+        <t>e.g. Europe/Warsaw — used by Lights auto</t>
       </text>
     </comment>
   </commentList>
@@ -375,57 +467,42 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Utility feed, generator, UPS, panel, breaker or PDU. If it is mounted in a rack, also list it in Devices with the same name</t>
+        <t>Same rack names as in Devices</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>utility, wall outlet, generator, UPS, panel, breaker, PDU, power strip, smart plug</t>
+        <t>Row name. Racks in the same row stand side by side</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Number with unit: 11 kVA, 16 A, 22 kW</t>
+        <t>Room name from the Rooms sheet (one room if empty)</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Name of the item above it in the chain</t>
+        <t>Order in the row: 1, 2, 3 …</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Feed letter: A or B</t>
+        <t>Default 42</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Rack it sits in or supplies (for PDUs)</t>
+        <t>19 (default) or 10 for a mini rack</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>e.g. 230 V, 400 V, 120 V</t>
+        <t>Aisle the rack front faces: A or B. Empty = rows alternate automatically (hot/cold aisle)</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>1 or 3</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>For single-phase items fed from a 3-phase supply: L1, L2 or L3</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>UPS only: runtime in minutes at the load you expect (from the vendor table)</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>UPS / battery cabinet only: usable battery energy in kWh</t>
+        <t>Design power for this rack, if known</t>
       </text>
     </comment>
   </commentList>
@@ -440,17 +517,57 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>VLAN id</t>
+        <t>Utility feed, generator, UPS, panel, breaker or PDU. If it is mounted in a rack, also list it in Devices with the same name</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>utility, wall outlet, generator, UPS, panel, breaker, PDU, power strip, smart plug</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>servers, storage, management, IoT, guest, AI fabric …</t>
+        <t>Number with unit: 11 kVA, 16 A, 22 kW</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Optional, e.g. 10.0.10.0/24</t>
+        <t>Name of the item above it in the chain</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Feed letter: A or B</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Rack it sits in or supplies (for PDUs)</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. 230 V, 400 V, 120 V</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>1 or 3</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>For single-phase items fed from a 3-phase supply: L1, L2 or L3</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>UPS only: runtime in minutes at the load you expect (from the vendor table)</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>UPS / battery cabinet only: usable battery energy in kWh</t>
       </text>
     </comment>
   </commentList>
@@ -463,19 +580,19 @@
     <author>template</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>CRAH, CRAC, in-row, rear-door, CDU, split AC</t>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>VLAN id</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Cooling capacity</t>
+        <t>servers, storage, management, IoT, guest, AI fabric …</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Rows or racks it cools, separated by ;</t>
+        <t>Optional, e.g. 10.0.10.0/24</t>
       </text>
     </comment>
   </commentList>
@@ -490,42 +607,37 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Short name you then use in Devices.model, e.g. "my-nas"</t>
+        <t>Site name from the Sites sheet</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>server, gpu_server, switch, storage, nas, mini_pc, sbc, patch_panel, pdu, ups, rack, crah, cdu, fire, generic …</t>
+        <t>Site name from the Sites sheet</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>dark fibre, wavelength, mpls, ip transit, vpn, replication</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Empty = no U (shelf)</t>
+        <t>Round trip. Empty = estimated from distance (fibre route ≈ 1.5 × great circle, 5 µs/km)</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>19 (default) or 10</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Rating of one PSU</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>front-to-back, back-to-front, side, none</t>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <t>e.g. "2x25G SFP28; 4x1G RJ45; 1x IPMI"</t>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <t>Category fields as JSON, e.g. {"va":1500,"runtime":[{"load_w":500,"minutes":12}]}</t>
+        <t>Typical load, 0–100</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>yes if a second path exists</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>free text</t>
       </text>
     </comment>
   </commentList>
@@ -538,24 +650,19 @@
     <author>template</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Date and time, e.g. 2026-10-01 14:00</t>
-      </text>
-    </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Device, rack, power item or sensor name; for a port use device:port, e.g. sw-core:SFP+1</t>
+        <t>CRAH, CRAC, in-row, rear-door, CDU, split AC</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>power_w, current_a, inlet_temp_c, outlet_temp_c, humidity_pct, link_mbps, port_errors, gpu_util_pct, tokens_per_s …</t>
+        <t>Cooling capacity</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Number</t>
+        <t>Rows or racks it cools, separated by ;</t>
       </text>
     </comment>
   </commentList>
@@ -851,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -905,74 +1012,88 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSV works too: one file per sheet (devices.csv, cables.csv, racks.csv, power.csv, networks.csv, cooling.csv, customdevices.csv, readings.csv) with the same column names.</t>
+          <t>Template v1.4 (2026-10-15): optional Sites sheet (coordinates, role, design kW/PUE) and Links sheet (site-to-site WAN) for the Globe view; Rooms.site.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CSV works too: one file per sheet (devices.csv, cables.csv, sites.csv, rooms.csv, links.csv, racks.csv, power.csv, networks.csv, cooling.csv, customdevices.csv, readings.csv) with the same column names.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Devices — what sits where. From the model name we fill in size, weight, power, airflow and the inside of the device.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cables — every power, network and storage cable, end to end. Enables the Cabling view (trace any cable), the Power view and the Network view.</t>
+          <t>Sites — where each data center is (coordinates). Enables the Globe view. Links — the WAN between sites: bandwidth, latency, protection.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Racks — which racks stand in which row. Without it, all racks from Devices are placed in one row.</t>
+          <t>Devices — what sits where. From the model name we fill in size, weight, power, airflow and the inside of the device.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Power — utility, UPS, panels, breakers and PDUs. Enables the power diagram, "what if feed A fails" and overload checks.</t>
+          <t>Cables — every power, network and storage cable, end to end. Enables the Cabling view (trace any cable), the Power view and the Network view.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Networks — your VLANs. Colours links in the Network view.</t>
+          <t>Racks — which racks stand in which row. Without it, all racks from Devices are placed in one row.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cooling — air conditioning and liquid cooling. Enables cooling-vs-heat checks and "what if AC-1 stops".</t>
+          <t>Power — utility, UPS, panels, breakers and PDUs. Enables the power diagram, "what if feed A fails" and overload checks.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Readings — history exported from your monitoring tool (Zabbix, SolarWinds, PRTG, Grafana …). Makes the simulation match your real room.</t>
+          <t>Networks — your VLANs. Colours links in the Network view.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cooling — air conditioning and liquid cooling. Enables cooling-vs-heat checks and "what if AC-1 stops".</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>Readings — history exported from your monitoring tool (Zabbix, SolarWinds, PRTG, Grafana …). Makes the simulation match your real room.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Unknown model names are fine: they become a plain box of the right height and you can identify them later.</t>
         </is>
@@ -984,6 +1105,269 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>capacity_kw</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>serves</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>AC-1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>CRAH</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Row A; Row B</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CRAH,CRAC,in-row,rear-door,CDU,split AC"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>height_u</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>width_in</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>depth_mm</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>weight_kg</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>psu_count</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>psu_w</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>idle_w</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>typical_w</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>max_w</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>airflow</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>inlet_max_c</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>ports</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>extra_json</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>my-nas</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>nas</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Acme</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>NAS-8</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="M2" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>front-to-back</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>2x10G SFP+; 2x1G RJ45</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>{"bays":"8x3.5"}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1858,80 +2242,155 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>room</t>
+          <t>site</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>length_m</t>
+          <t>city</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>width_m</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>height_m</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>raised_floor_mm</t>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>lon</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>lighting_w</t>
+          <t>timezone</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>timezone</t>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>provider</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>it_kw</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>pue</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Hall 1</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>8</v>
+          <t>FRA-1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Frankfurt</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>3.2</v>
+        <v>50.1109</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>600</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>580</v>
+        <v>8.6821</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Europe/Berlin</t>
+        </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Europe/Warsaw</t>
-        </is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>SIN-1</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1.3521</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>103.8198</v>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Asia/Singapore</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>dr</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>colo</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>1.35</v>
       </c>
     </row>
   </sheetData>
@@ -1941,6 +2400,105 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>room</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>length_m</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>width_m</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>height_m</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>raised_floor_mm</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>lighting_w</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>timezone</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Hall 1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>FRA-1</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>580</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Europe/Warsaw</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2114,7 +2672,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2444,7 +3002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2535,262 +3093,96 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>capacity_kw</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>serves</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>AC-1</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>CRAH</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Row A; Row B</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"CRAH,CRAC,in-row,rear-door,CDU,split AC"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>site_a</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>site_b</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>brand</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>model</t>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>bandwidth_gbps</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>height_u</t>
+          <t>latency_ms</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>width_in</t>
+          <t>utilization_pct</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>depth_mm</t>
+          <t>protected</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>weight_kg</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>psu_count</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>psu_w</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>idle_w</t>
-        </is>
-      </c>
-      <c r="L1" s="4" t="inlineStr">
-        <is>
-          <t>typical_w</t>
-        </is>
-      </c>
-      <c r="M1" s="4" t="inlineStr">
-        <is>
-          <t>max_w</t>
-        </is>
-      </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>airflow</t>
-        </is>
-      </c>
-      <c r="O1" s="4" t="inlineStr">
-        <is>
-          <t>inlet_max_c</t>
-        </is>
-      </c>
-      <c r="P1" s="4" t="inlineStr">
-        <is>
-          <t>ports</t>
-        </is>
-      </c>
-      <c r="Q1" s="4" t="inlineStr">
-        <is>
-          <t>extra_json</t>
+          <t>carrier</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>my-nas</t>
+          <t>FRA-1</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>nas</t>
+          <t>SIN-1</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Acme</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>NAS-8</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>2</v>
-      </c>
+          <t>wavelength</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>450</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="5" t="n">
-        <v>250</v>
-      </c>
-      <c r="K2" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="L2" s="5" t="n">
-        <v>60</v>
-      </c>
-      <c r="M2" s="5" t="n">
-        <v>120</v>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>front-to-back</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="P2" s="5" t="inlineStr">
-        <is>
-          <t>2x10G SFP+; 2x1G RJ45</t>
-        </is>
-      </c>
-      <c r="Q2" s="5" t="inlineStr">
-        <is>
-          <t>{"bays":"8x3.5"}</t>
-        </is>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DC template download v1.5 (Liquid sheet, Cooling.chilled_from, Racks.depth_mm): xlsx from dc-import, twelve sheets, template page en/de/zh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/dc/downloads/dc-import-template.xlsx
+++ b/public/dc/downloads/dc-import-template.xlsx
@@ -17,8 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Networks" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Links" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cooling" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CustomDevices" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readings" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquid" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CustomDevices" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readings" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -237,42 +238,57 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Short name you then use in Devices.model, e.g. "my-nas"</t>
+        <t>Loop name, e.g. "DLC-1"</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>server, gpu_server, switch, storage, nas, mini_pc, sbc, patch_panel, pdu, ups, rack, crah, cdu, fire, generic …</t>
+        <t>dlc (direct-to-chip), rdhx (rear-door heat exchanger), immersion</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>CDU name from the Devices sheet (model from the catalog), empty for facility-water RDHx</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Heat the loop can reject</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Empty = no U (shelf)</t>
+        <t>Supply temperature °C</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>19 (default) or 10</t>
+        <t>Return temperature °C</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Flow in litres per minute</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>water-glycol 25%, PG25, dielectric …</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Racks or rows on this loop, e.g. "R01-R08" or "Row A"</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Rating of one PSU</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>front-to-back, back-to-front, side, none</t>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <t>e.g. "2x25G SFP28; 4x1G RJ45; 1x IPMI"</t>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <t>Category fields as JSON, e.g. {"va":1500,"runtime":[{"load_w":500,"minutes":12}]}</t>
+        <t>Facility loop or chiller feeding the CDU, e.g. "FWS-1"</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Manifold name, e.g. "MAN-A1" (leak what-if isolates per manifold)</t>
       </text>
     </comment>
   </commentList>
@@ -287,6 +303,56 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
+        <t>Short name you then use in Devices.model, e.g. "my-nas"</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>server, gpu_server, switch, storage, nas, mini_pc, sbc, patch_panel, pdu, ups, rack, crah, cdu, fire, generic …</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Empty = no U (shelf)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>19 (default) or 10</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Rating of one PSU</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>front-to-back, back-to-front, side, none</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>e.g. "2x25G SFP28; 4x1G RJ45; 1x IPMI"</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Category fields as JSON, e.g. {"va":1500,"runtime":[{"load_w":500,"minutes":12}]}</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
         <t>Date and time, e.g. 2026-10-01 14:00</t>
       </text>
     </comment>
@@ -492,15 +558,20 @@
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
+        <t>Usable rack depth in mm (fit checks against device depth); empty = no depth check</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
         <t>19 (default) or 10 for a mini rack</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Aisle the rack front faces: A or B. Empty = rows alternate automatically (hot/cold aisle)</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Design power for this rack, if known</t>
       </text>
@@ -663,6 +734,11 @@
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>Rows or racks it cools, separated by ;</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Chilled-water source for CRAH / chilled-water units, e.g. "CH-1" (empty = DX unit)</t>
       </text>
     </comment>
   </commentList>
@@ -958,7 +1034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -1019,81 +1095,95 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CSV works too: one file per sheet (devices.csv, cables.csv, sites.csv, rooms.csv, links.csv, racks.csv, power.csv, networks.csv, cooling.csv, customdevices.csv, readings.csv) with the same column names.</t>
+          <t>Template v1.5 (2026-10-15): optional Liquid sheet (DLC / rear-door / immersion loops: CDU, capacity, temperatures, flow, served racks, manifold); Cooling.chilled_from (chilled-water source; empty = DX); Racks.depth_mm.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CSV works too: one file per sheet (devices.csv, cables.csv, sites.csv, rooms.csv, links.csv, racks.csv, power.csv, networks.csv, cooling.csv, liquid.csv, customdevices.csv, readings.csv) with the same column names.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Sites — where each data center is (coordinates). Enables the Globe view. Links — the WAN between sites: bandwidth, latency, protection.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Devices — what sits where. From the model name we fill in size, weight, power, airflow and the inside of the device.</t>
+          <t>Sites — where each data center is (coordinates). Enables the Globe view. Links — the WAN between sites: bandwidth, latency, protection.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cables — every power, network and storage cable, end to end. Enables the Cabling view (trace any cable), the Power view and the Network view.</t>
+          <t>Devices — what sits where. From the model name we fill in size, weight, power, airflow and the inside of the device.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Racks — which racks stand in which row. Without it, all racks from Devices are placed in one row.</t>
+          <t>Cables — every power, network and storage cable, end to end. Enables the Cabling view (trace any cable), the Power view and the Network view.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Power — utility, UPS, panels, breakers and PDUs. Enables the power diagram, "what if feed A fails" and overload checks.</t>
+          <t>Racks — which racks stand in which row. Without it, all racks from Devices are placed in one row.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Networks — your VLANs. Colours links in the Network view.</t>
+          <t>Power — utility, UPS, panels, breakers and PDUs. Enables the power diagram, "what if feed A fails" and overload checks.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cooling — air conditioning and liquid cooling. Enables cooling-vs-heat checks and "what if AC-1 stops".</t>
+          <t>Networks — your VLANs. Colours links in the Network view.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Readings — history exported from your monitoring tool (Zabbix, SolarWinds, PRTG, Grafana …). Makes the simulation match your real room.</t>
+          <t>Cooling — air conditioning units. Enables cooling-vs-heat checks and "what if AC-1 stops".</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Liquid — direct-to-chip, rear-door and immersion loops with their CDUs and manifolds. Enables the liquid heat balance and "what if a manifold leaks".</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
+        <is>
+          <t>Readings — history exported from your monitoring tool (Zabbix, SolarWinds, PRTG, Grafana …). Makes the simulation match your real room.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Unknown model names are fine: they become a plain box of the right height and you can identify them later.</t>
         </is>
@@ -1110,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1118,6 +1208,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1144,6 +1235,11 @@
       <c r="E1" s="4" t="inlineStr">
         <is>
           <t>model</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>chilled_from</t>
         </is>
       </c>
     </row>
@@ -1180,6 +1276,140 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>loop</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>cdu</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>capacity_kw</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>supply_c</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>return_c</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>flow_lpm</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>coolant</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>serves</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>manifold</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>DLC-1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>dlc</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>CDU-1</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>PG25</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>R01-R08</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>FWS-1</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>MAN-A1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1367,7 +1597,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2504,7 +2734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2513,8 +2743,9 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2545,15 +2776,20 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>depth_mm</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>width_in</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>front_faces</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>max_kw</t>
         </is>
@@ -2582,14 +2818,17 @@
         <v>42</v>
       </c>
       <c r="F2" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="I2" s="5" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2616,14 +2855,17 @@
         <v>42</v>
       </c>
       <c r="F3" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G3" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="I3" s="5" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2650,14 +2892,17 @@
         <v>42</v>
       </c>
       <c r="F4" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="I4" s="5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>